<commit_message>
docs(homologacao): pacote de evidencias completo — 21 passos, logs do PayGo e os 33 callbacks recebidos
O passo 50 exigia Callback/Insert MAIS o POST recebido. Ate agora so tinhamos o
200 do cadastro: o log do endpoint mora em arquivo proprio (paygo-callback.log),
nao no access.log, e por isso passava por nao existir. Chegaram 33 POSTs.

Ressalva registrada no LEIA-ME: a venda do passo 06 e anterior ao cadastro da URL
e nao gerou callback; a prova vem das outras vendas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
EOF
)
</commit_message>
<xml_diff>
--- a/docs/evidencias-controlpay/Planilha de testes v20260703 - PREENCHIDA.xlsx
+++ b/docs/evidencias-controlpay/Planilha de testes v20260703 - PREENCHIDA.xlsx
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E66"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1796875" defaultRowHeight="15.5"/>
   <cols>
     <col width="12.54296875" customWidth="1" style="1" min="1" max="1"/>
@@ -700,6 +700,7 @@
     <col width="9.1796875" customWidth="1" style="1" min="6" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
@@ -1361,8 +1362,16 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="5" t="n"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>167602</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Queda de energia durante a venda: PC desligado no botao quando o pinpad pediu o cartao. Ao religar, a reconciliacao fechou a linha como recusado ("religamento: Pagamento Recusado"); nenhuma venda foi gravada (venda_id NULL). Nunca ficou paga.</t>
+        </is>
+      </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Queda energia</t>
@@ -1929,12 +1938,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>200 OK</t>
+          <t>167572</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Callback/Insert tipo 1 UrlRetorno -&gt; https://erp.americandaybrasil.com.br/paygo-callback</t>
+          <t>Callback/Insert cadastrado (200 OK) para https://erp.americandaybrasil.com.br/paygo-callback e POSTs RECEBIDOS: 33 notificacoes da PayGo (origem 191.232.70.197) em 24/08/2026, cada uma com intencaoVendaId na query. Evidencia em p50-callbacks-recebidos.log. Exemplos: 167572 (passo 19), 167575 (passo 30), 167576 (passo 45), 167577 (passo 46), 167598 (passo 52), 167602 (passo 24). Observacao: a venda do passo 06 (167513) e anterior ao cadastro da URL, por isso nao gerou callback.</t>
         </is>
       </c>
       <c r="E61" s="34" t="n"/>
@@ -1973,8 +1982,16 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="C63" s="4" t="n"/>
-      <c r="D63" s="5" t="n"/>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>167598</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Venda PIX de R$ 500,00 com Esc na tela do QR: OPERACAO CANCELADA.</t>
+        </is>
+      </c>
       <c r="E63" s="21" t="inlineStr">
         <is>
           <t>QR Code</t>

</xml_diff>

<commit_message>
docs(homologacao): reenvio 25/08 — retestes pedidos pela analise da SETIS
A analise pediu: passos 6 e 7 com o cartao inserido no chip (tinham saido por
aproximacao) e passos 17, 18, 20 e 22 na adquirente C6 PAY (tinham saido na REDE).

Os passos 49 e 50 foram trocados junto, sem terem sido pedidos: os dois
referenciam a venda do passo 6, que mudou de numero no reteste. Deixa-los como
estavam apontaria para uma venda que nao e mais a do passo -- e voltaria pelo
mesmo motivo.

A insercao no chip esta provada em dois lugares independentes: o comprovante traz
o prefixo C- na linha do cartao (aproximacao imprime L-), e o log do PayGo tem
PW_iPPGoOnChip com PWRET_OK oito segundos apos o inicio de cada venda -- 10:24:49
no passo 6 e 10:31:48 no passo 7.

Logs regerados cobrindo 21 a 25/08.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evidencias-controlpay/Planilha de testes v20260703 - PREENCHIDA.xlsx
+++ b/docs/evidencias-controlpay/Planilha de testes v20260703 - PREENCHIDA.xlsx
@@ -946,12 +946,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>167658</t>
+          <t>167726</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Venda de R$ 10,00 no credito, aprovada. E a venda consultada no passo 49 e notificada no callback do passo 50.</t>
+          <t>Venda de R$ 10,00 no credito, com o cartao INSERIDO no chip (adquirente C6 PAY). O comprovante traz o prefixo C- na linha do cartao, que identifica a leitura por chip. E a venda consultada no passo 49 e notificada no callback do passo 50.</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>167659</t>
+          <t>167733</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Venda de R$ 10,00 no debito, aprovada.</t>
+          <t>Venda de R$ 10,00 no debito, com o cartao INSERIDO no chip (adquirente C6 PAY). O comprovante traz o prefixo C- na linha do cartao.</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>167566</t>
+          <t>167730</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Venda de R$ 1,00 no credito, aprovada, para ser cancelada no passo 22.</t>
+          <t>Venda de R$ 1,00 no credito pela adquirente C6 PAY, aprovada, para ser cancelada no passo 22.</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>167567</t>
+          <t>167731</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Venda de R$ 2,00 no credito, aprovada, para ser cancelada no passo 20.</t>
+          <t>Venda de R$ 2,00 no credito pela adquirente C6 PAY, aprovada, para ser cancelada no passo 20.</t>
         </is>
       </c>
       <c r="E29" s="33" t="n"/>
@@ -1276,12 +1276,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>167567</t>
+          <t>167731</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Cancelamento da venda do passo 18 (R$ 2,00), aprovado, com comprovante de estorno.</t>
+          <t>Cancelamento da venda do passo 18 (R$ 2,00, C6 PAY), aprovado, com comprovante de estorno.</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
@@ -1326,12 +1326,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>167566</t>
+          <t>167730</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Cancelamento da venda do passo 17 (R$ 1,00), aprovado, com comprovante de estorno.</t>
+          <t>Cancelamento da venda do passo 17 (R$ 1,00, C6 PAY), aprovado, com comprovante de estorno.</t>
         </is>
       </c>
       <c r="E33" s="33" t="n"/>
@@ -1915,12 +1915,12 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>167658</t>
+          <t>167726</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>IntencaoVenda/GetById da venda do passo 06: status 10 (Creditado), valor 10,00. JSON em p49-intencao-167658.json.</t>
+          <t>IntencaoVenda/GetById da venda do passo 06: status 10 (Creditado), valor 10,00. JSON em p49-intencao-167726.json.</t>
         </is>
       </c>
       <c r="E60" s="33" t="n"/>
@@ -1938,12 +1938,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>167658</t>
+          <t>167726</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Callback/Insert cadastrado (200 OK) e POST recebido. A venda do passo 06 gerou a notificacao em 24/08 as 17:12:15, com o intencaoVendaId na query. Log completo em p50-callbacks-recebidos.log, com 38 notificacoes recebidas no total.</t>
+          <t>Callback/Insert cadastrado (200 OK) e POST recebido. A venda do passo 06 gerou a notificacao em 25/08 as 10:25:18, com o intencaoVendaId na query. Log completo em p50-callbacks-recebidos.log, com 49 notificacoes recebidas no total.</t>
         </is>
       </c>
       <c r="E61" s="34" t="n"/>

</xml_diff>